<commit_message>
feat(checkout): phan tich + gen TC Camera + AP (ban revise 0306)
- Phan tich DOC-CK-04 (Chucnangcheckout_0306.xlsx): them 2 sub-module CAMERA (20 SC) + AP (18 SC). UltraFast/CKCOMMON/Internet khong doi.
- Camera/AP tai dung CKCOMMON cho field validation, chi viet phan dac thu.
- Gen 2 sheet TC: Checkout_Camera (16 TC) + Checkout_AP (14 TC).
- 8 TC BLOCKED (highlight cam) cho clarification chua xac nhan: CLA-CAMERA-001, CLA-AP-001, CLA-AP-002 + voucher chua implement.
- Cap nhat MEMORY/traceability/risk/scenario_map + CLAUDE.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.0.xlsx
+++ b/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.0.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_Common" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_Internet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_Camera" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_AP" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +49,20 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -65,8 +79,18 @@
         <fgColor rgb="00A9D08E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A4C2F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -121,11 +145,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -146,6 +214,44 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -599,19 +705,19 @@
           <t>Round 1</t>
         </is>
       </c>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="11" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Kết Quả Thực Hiện</t>
@@ -639,16 +745,16 @@
           <t>Nhóm 1: Hiển thị tổng thể &amp; Điều hướng</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="10" t="n"/>
+      <c r="I9" s="10" t="n"/>
+      <c r="J9" s="10" t="n"/>
+      <c r="K9" s="10" t="n"/>
+      <c r="L9" s="11" t="n"/>
     </row>
     <row r="10" ht="255" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -941,16 +1047,16 @@
           <t>Nhóm 2: Block Sản phẩm dịch vụ đã chọn</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="10" t="n"/>
+      <c r="I16" s="10" t="n"/>
+      <c r="J16" s="10" t="n"/>
+      <c r="K16" s="10" t="n"/>
+      <c r="L16" s="11" t="n"/>
     </row>
     <row r="17" ht="135" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -1003,16 +1109,16 @@
           <t>Nhóm 3: Block Thông tin cá nhân — Họ tên</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
-      <c r="L18" s="5" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="10" t="n"/>
+      <c r="J18" s="10" t="n"/>
+      <c r="K18" s="10" t="n"/>
+      <c r="L18" s="11" t="n"/>
     </row>
     <row r="19" ht="180" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
@@ -1255,16 +1361,16 @@
           <t>Nhóm 4: Block Thông tin cá nhân — Số điện thoại</t>
         </is>
       </c>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="5" t="n"/>
-      <c r="K24" s="5" t="n"/>
-      <c r="L24" s="5" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="10" t="n"/>
+      <c r="I24" s="10" t="n"/>
+      <c r="J24" s="10" t="n"/>
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="11" t="n"/>
     </row>
     <row r="25" ht="135" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
@@ -1550,16 +1656,16 @@
           <t>Nhóm 5: Block Thông tin cá nhân — Email (chỉ Hyperfast/UltraFast)</t>
         </is>
       </c>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="5" t="n"/>
-      <c r="L31" s="5" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="10" t="n"/>
+      <c r="H31" s="10" t="n"/>
+      <c r="I31" s="10" t="n"/>
+      <c r="J31" s="10" t="n"/>
+      <c r="K31" s="10" t="n"/>
+      <c r="L31" s="11" t="n"/>
     </row>
     <row r="32" ht="120" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
@@ -1752,16 +1858,16 @@
           <t>Nhóm 6: Block Địa chỉ lắp đặt — Tỉnh/Thành phố &amp; pre-fill</t>
         </is>
       </c>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="5" t="n"/>
-      <c r="L36" s="5" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="n"/>
+      <c r="H36" s="10" t="n"/>
+      <c r="I36" s="10" t="n"/>
+      <c r="J36" s="10" t="n"/>
+      <c r="K36" s="10" t="n"/>
+      <c r="L36" s="11" t="n"/>
     </row>
     <row r="37" ht="135" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
@@ -2092,16 +2198,16 @@
           <t>Nhóm 7: Block Địa chỉ lắp đặt — Phường/Xã &amp; kiểm tra chính sách giá</t>
         </is>
       </c>
-      <c r="C44" s="5" t="n"/>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="5" t="n"/>
-      <c r="I44" s="5" t="n"/>
-      <c r="J44" s="5" t="n"/>
-      <c r="K44" s="5" t="n"/>
-      <c r="L44" s="5" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="10" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="10" t="n"/>
+      <c r="H44" s="10" t="n"/>
+      <c r="I44" s="10" t="n"/>
+      <c r="J44" s="10" t="n"/>
+      <c r="K44" s="10" t="n"/>
+      <c r="L44" s="11" t="n"/>
     </row>
     <row r="45" ht="105" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
@@ -2341,16 +2447,16 @@
           <t>Nhóm 8: Block Địa chỉ lắp đặt — Tên đường</t>
         </is>
       </c>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
-      <c r="J50" s="5" t="n"/>
-      <c r="K50" s="5" t="n"/>
-      <c r="L50" s="5" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="10" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="10" t="n"/>
+      <c r="H50" s="10" t="n"/>
+      <c r="I50" s="10" t="n"/>
+      <c r="J50" s="10" t="n"/>
+      <c r="K50" s="10" t="n"/>
+      <c r="L50" s="11" t="n"/>
     </row>
     <row r="51" ht="105" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
@@ -2450,16 +2556,16 @@
           <t>Nhóm 9: Block Địa chỉ lắp đặt — Số nhà (radio Nhà riêng/Chung cư: đặc thù dịch vụ thiết bị; Chung cư DEFERRED)</t>
         </is>
       </c>
-      <c r="C53" s="5" t="n"/>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="5" t="n"/>
-      <c r="I53" s="5" t="n"/>
-      <c r="J53" s="5" t="n"/>
-      <c r="K53" s="5" t="n"/>
-      <c r="L53" s="5" t="n"/>
+      <c r="C53" s="10" t="n"/>
+      <c r="D53" s="10" t="n"/>
+      <c r="E53" s="10" t="n"/>
+      <c r="F53" s="10" t="n"/>
+      <c r="G53" s="10" t="n"/>
+      <c r="H53" s="10" t="n"/>
+      <c r="I53" s="10" t="n"/>
+      <c r="J53" s="10" t="n"/>
+      <c r="K53" s="10" t="n"/>
+      <c r="L53" s="11" t="n"/>
     </row>
     <row r="54" ht="195" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
@@ -2603,16 +2709,16 @@
           <t>Nhóm 10: Block Địa chỉ lắp đặt — Ghi chú</t>
         </is>
       </c>
-      <c r="C57" s="5" t="n"/>
-      <c r="D57" s="5" t="n"/>
-      <c r="E57" s="5" t="n"/>
-      <c r="F57" s="5" t="n"/>
-      <c r="G57" s="5" t="n"/>
-      <c r="H57" s="5" t="n"/>
-      <c r="I57" s="5" t="n"/>
-      <c r="J57" s="5" t="n"/>
-      <c r="K57" s="5" t="n"/>
-      <c r="L57" s="5" t="n"/>
+      <c r="C57" s="10" t="n"/>
+      <c r="D57" s="10" t="n"/>
+      <c r="E57" s="10" t="n"/>
+      <c r="F57" s="10" t="n"/>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="10" t="n"/>
+      <c r="I57" s="10" t="n"/>
+      <c r="J57" s="10" t="n"/>
+      <c r="K57" s="10" t="n"/>
+      <c r="L57" s="11" t="n"/>
     </row>
     <row r="58" ht="150" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
@@ -2667,16 +2773,16 @@
           <t>Nhóm 11: Popup Địa chỉ hành chính cũ (3 cấp → 2 cấp)</t>
         </is>
       </c>
-      <c r="C59" s="5" t="n"/>
-      <c r="D59" s="5" t="n"/>
-      <c r="E59" s="5" t="n"/>
-      <c r="F59" s="5" t="n"/>
-      <c r="G59" s="5" t="n"/>
-      <c r="H59" s="5" t="n"/>
-      <c r="I59" s="5" t="n"/>
-      <c r="J59" s="5" t="n"/>
-      <c r="K59" s="5" t="n"/>
-      <c r="L59" s="5" t="n"/>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="10" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="10" t="n"/>
+      <c r="G59" s="10" t="n"/>
+      <c r="H59" s="10" t="n"/>
+      <c r="I59" s="10" t="n"/>
+      <c r="J59" s="10" t="n"/>
+      <c r="K59" s="10" t="n"/>
+      <c r="L59" s="11" t="n"/>
     </row>
     <row r="60" ht="120" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
@@ -2956,16 +3062,16 @@
           <t>Nhóm 12: Block Thông tin khách hàng</t>
         </is>
       </c>
-      <c r="C66" s="5" t="n"/>
-      <c r="D66" s="5" t="n"/>
-      <c r="E66" s="5" t="n"/>
-      <c r="F66" s="5" t="n"/>
-      <c r="G66" s="5" t="n"/>
-      <c r="H66" s="5" t="n"/>
-      <c r="I66" s="5" t="n"/>
-      <c r="J66" s="5" t="n"/>
-      <c r="K66" s="5" t="n"/>
-      <c r="L66" s="5" t="n"/>
+      <c r="C66" s="10" t="n"/>
+      <c r="D66" s="10" t="n"/>
+      <c r="E66" s="10" t="n"/>
+      <c r="F66" s="10" t="n"/>
+      <c r="G66" s="10" t="n"/>
+      <c r="H66" s="10" t="n"/>
+      <c r="I66" s="10" t="n"/>
+      <c r="J66" s="10" t="n"/>
+      <c r="K66" s="10" t="n"/>
+      <c r="L66" s="11" t="n"/>
     </row>
     <row r="67" ht="120" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
@@ -3109,16 +3215,16 @@
           <t>Nhóm 13: Block Phương thức thanh toán</t>
         </is>
       </c>
-      <c r="C70" s="5" t="n"/>
-      <c r="D70" s="5" t="n"/>
-      <c r="E70" s="5" t="n"/>
-      <c r="F70" s="5" t="n"/>
-      <c r="G70" s="5" t="n"/>
-      <c r="H70" s="5" t="n"/>
-      <c r="I70" s="5" t="n"/>
-      <c r="J70" s="5" t="n"/>
-      <c r="K70" s="5" t="n"/>
-      <c r="L70" s="5" t="n"/>
+      <c r="C70" s="10" t="n"/>
+      <c r="D70" s="10" t="n"/>
+      <c r="E70" s="10" t="n"/>
+      <c r="F70" s="10" t="n"/>
+      <c r="G70" s="10" t="n"/>
+      <c r="H70" s="10" t="n"/>
+      <c r="I70" s="10" t="n"/>
+      <c r="J70" s="10" t="n"/>
+      <c r="K70" s="10" t="n"/>
+      <c r="L70" s="11" t="n"/>
     </row>
     <row r="71" ht="120" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
@@ -3354,16 +3460,16 @@
           <t>Nhóm 14: Block Thông tin thanh toán &amp; Mã ưu đãi</t>
         </is>
       </c>
-      <c r="C76" s="5" t="n"/>
-      <c r="D76" s="5" t="n"/>
-      <c r="E76" s="5" t="n"/>
-      <c r="F76" s="5" t="n"/>
-      <c r="G76" s="5" t="n"/>
-      <c r="H76" s="5" t="n"/>
-      <c r="I76" s="5" t="n"/>
-      <c r="J76" s="5" t="n"/>
-      <c r="K76" s="5" t="n"/>
-      <c r="L76" s="5" t="n"/>
+      <c r="C76" s="10" t="n"/>
+      <c r="D76" s="10" t="n"/>
+      <c r="E76" s="10" t="n"/>
+      <c r="F76" s="10" t="n"/>
+      <c r="G76" s="10" t="n"/>
+      <c r="H76" s="10" t="n"/>
+      <c r="I76" s="10" t="n"/>
+      <c r="J76" s="10" t="n"/>
+      <c r="K76" s="10" t="n"/>
+      <c r="L76" s="11" t="n"/>
     </row>
     <row r="77" ht="135" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
@@ -3646,16 +3752,16 @@
           <t>Nhóm 15: Luồng thanh toán</t>
         </is>
       </c>
-      <c r="C83" s="5" t="n"/>
-      <c r="D83" s="5" t="n"/>
-      <c r="E83" s="5" t="n"/>
-      <c r="F83" s="5" t="n"/>
-      <c r="G83" s="5" t="n"/>
-      <c r="H83" s="5" t="n"/>
-      <c r="I83" s="5" t="n"/>
-      <c r="J83" s="5" t="n"/>
-      <c r="K83" s="5" t="n"/>
-      <c r="L83" s="5" t="n"/>
+      <c r="C83" s="10" t="n"/>
+      <c r="D83" s="10" t="n"/>
+      <c r="E83" s="10" t="n"/>
+      <c r="F83" s="10" t="n"/>
+      <c r="G83" s="10" t="n"/>
+      <c r="H83" s="10" t="n"/>
+      <c r="I83" s="10" t="n"/>
+      <c r="J83" s="10" t="n"/>
+      <c r="K83" s="10" t="n"/>
+      <c r="L83" s="11" t="n"/>
     </row>
     <row r="84" ht="150" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
@@ -4083,16 +4189,16 @@
           <t>Nhóm 16: Màn hình Hoàn tất đơn hàng</t>
         </is>
       </c>
-      <c r="C93" s="5" t="n"/>
-      <c r="D93" s="5" t="n"/>
-      <c r="E93" s="5" t="n"/>
-      <c r="F93" s="5" t="n"/>
-      <c r="G93" s="5" t="n"/>
-      <c r="H93" s="5" t="n"/>
-      <c r="I93" s="5" t="n"/>
-      <c r="J93" s="5" t="n"/>
-      <c r="K93" s="5" t="n"/>
-      <c r="L93" s="5" t="n"/>
+      <c r="C93" s="10" t="n"/>
+      <c r="D93" s="10" t="n"/>
+      <c r="E93" s="10" t="n"/>
+      <c r="F93" s="10" t="n"/>
+      <c r="G93" s="10" t="n"/>
+      <c r="H93" s="10" t="n"/>
+      <c r="I93" s="10" t="n"/>
+      <c r="J93" s="10" t="n"/>
+      <c r="K93" s="10" t="n"/>
+      <c r="L93" s="11" t="n"/>
     </row>
     <row r="94" ht="105" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
@@ -4327,16 +4433,16 @@
           <t>Nhóm 17: Empty/Error state, Quyền truy cập &amp; Mobile (Mandatory)</t>
         </is>
       </c>
-      <c r="C99" s="5" t="n"/>
-      <c r="D99" s="5" t="n"/>
-      <c r="E99" s="5" t="n"/>
-      <c r="F99" s="5" t="n"/>
-      <c r="G99" s="5" t="n"/>
-      <c r="H99" s="5" t="n"/>
-      <c r="I99" s="5" t="n"/>
-      <c r="J99" s="5" t="n"/>
-      <c r="K99" s="5" t="n"/>
-      <c r="L99" s="5" t="n"/>
+      <c r="C99" s="10" t="n"/>
+      <c r="D99" s="10" t="n"/>
+      <c r="E99" s="10" t="n"/>
+      <c r="F99" s="10" t="n"/>
+      <c r="G99" s="10" t="n"/>
+      <c r="H99" s="10" t="n"/>
+      <c r="I99" s="10" t="n"/>
+      <c r="J99" s="10" t="n"/>
+      <c r="K99" s="10" t="n"/>
+      <c r="L99" s="11" t="n"/>
     </row>
     <row r="100" ht="150" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
@@ -4648,19 +4754,19 @@
           <t>Round 1</t>
         </is>
       </c>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="11" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Kết Quả Thực Hiện</t>
@@ -4688,16 +4794,16 @@
           <t>Nhóm 1: Hiển thị tổng thể &amp; Điều hướng 3 bước</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="10" t="n"/>
+      <c r="I9" s="10" t="n"/>
+      <c r="J9" s="10" t="n"/>
+      <c r="K9" s="10" t="n"/>
+      <c r="L9" s="11" t="n"/>
     </row>
     <row r="10" ht="150" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -4840,16 +4946,16 @@
           <t>Nhóm 2: Bước 1 — Thông tin đăng ký</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
+      <c r="H13" s="10" t="n"/>
+      <c r="I13" s="10" t="n"/>
+      <c r="J13" s="10" t="n"/>
+      <c r="K13" s="10" t="n"/>
+      <c r="L13" s="11" t="n"/>
     </row>
     <row r="14" ht="120" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -5084,16 +5190,16 @@
           <t>Nhóm 3: Bước 2 — Thanh toán (trả trước/trả sau, giá động)</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="10" t="n"/>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="11" t="n"/>
     </row>
     <row r="20" ht="135" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -5374,16 +5480,16 @@
           <t>Nhóm 4: Bước 3 — Hoàn tất đơn hàng</t>
         </is>
       </c>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="5" t="n"/>
-      <c r="K26" s="5" t="n"/>
-      <c r="L26" s="5" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
+      <c r="J26" s="10" t="n"/>
+      <c r="K26" s="10" t="n"/>
+      <c r="L26" s="11" t="n"/>
     </row>
     <row r="27" ht="120" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
@@ -5528,16 +5634,16 @@
           <t>Nhóm 5: Mobile (Mandatory)</t>
         </is>
       </c>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="5" t="n"/>
-      <c r="L30" s="5" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="10" t="n"/>
+      <c r="J30" s="10" t="n"/>
+      <c r="K30" s="10" t="n"/>
+      <c r="L30" s="11" t="n"/>
     </row>
     <row r="31" ht="120" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
@@ -5603,4 +5709,1702 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A3:L32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="3">
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Mã chức năng:</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>TC_CAMERA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Tên chức năng:</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Đăng ký dịch vụ Camera — Checkout (chu kỳ + COD + địa chỉ lắp đặt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>QC/AI</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Testcase ID</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Mức Độ Ưu Tiên</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Nội Dung Test</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Điều Kiện / Dữ Liệu Test</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Các Bước Thực Hiện</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Kết Quả Mong Đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>Có thể
+Tự Động Hóa</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>Round 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>Kết Quả Thực Hiện</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>Người Thực Hiện</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>ID Bugs</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>Ghi Chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Lưu ý: Field validation (Họ tên, SĐT, Email, dropdown địa chỉ Tỉnh/Phường/Đường, popup Địa chỉ hành chính cũ, danh sách Phương thức thanh toán, luồng OTP) dùng chung — xem sheet Checkout_Common (TC_CKCOMMON). Sheet này chỉ kiểm tra phần ĐẶC THÙ dịch vụ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 1: Hiển thị tổng thể &amp; Điều hướng vào Checkout (chu kỳ + số lượng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B11" s="18">
+        <f>IF(D11="","",$D$3&amp;"."&amp;COUNTA($D$10:D11)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị tổng thể màn Checkout Camera (2 bước)</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>Đã chọn gói Camera ở màn Chi tiết</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát tiến trình và bố cục màn checkout Camera</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Header 2 bước: "Thanh toán" (xanh dương) → "Hoàn tất đơn hàng" (xám); hiển thị đủ block: Sản phẩm dịch vụ đã chọn, Thông tin cá nhân, Địa chỉ lắp đặt, Phương thức thanh toán, Thông tin khách hàng, Thông tin thanh toán</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <f>IF(D12="","",$D$3&amp;"."&amp;COUNTA($D$10:D12)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra chọn chu kỳ + số lượng rồi Mua ngay điều hướng sang Checkout</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>Ở màn Chi tiết gói Camera</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>1. Chọn chu kỳ bất kỳ + số lượng
+2. Click button "Mua ngay"</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Điều hướng sang màn Thanh toán; load đúng tên gói, chu kỳ, số lượng, số tiền như đã chọn ở Chi tiết</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B13" s="18">
+        <f>IF(D13="","",$D$3&amp;"."&amp;COUNTA($D$10:D13)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra đổi số lượng thì số tiền cập nhật đúng trên checkout</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>Ở Chi tiết chọn số lượng &gt; 1</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>1. Chọn số lượng &gt; 1
+2. Mua ngay sang checkout
+3. Đối chiếu số tiền</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Số tiền trên checkout = đơn giá × số lượng theo chu kỳ đã chọn (itemized: dòng Camera + dòng Gói Cloud)</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 2: Block Sản phẩm &amp; Thông tin thanh toán (đặc thù Camera)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B15" s="18">
+        <f>IF(D15="","",$D$3&amp;"."&amp;COUNTA($D$10:D15)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Sản phẩm dịch vụ đã chọn load đúng thông tin Camera</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Camera</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block "Sản phẩm dịch vụ đã chọn"</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Load đúng tên gói (vd Camera SE S2), dòng Cloud (vd Cloud 3 ngày), chu kỳ (vd 6 tháng), số lượng (x1), số tiền</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B16" s="18">
+        <f>IF(D16="","",$D$3&amp;"."&amp;COUNTA($D$10:D16)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Thông tin thanh toán itemized + Cần thanh toán</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Camera</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block "Thông tin thanh toán"
+2. Đối chiếu dòng Cần thanh toán</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Itemized đúng (vd "Camera SE S2 - 1 cái: 600.000đ", "Gói Cloud 3D - 6 tháng: 240.000đ"); "Cần thanh toán" = tổng tiền (vd 840.000đ)</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 3: Phương thức thanh toán &amp; Thông tin khách hàng (đặc thù Camera)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B18" s="18">
+        <f>IF(D18="","",$D$3&amp;"."&amp;COUNTA($D$10:D18)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra Camera CÓ phương thức COD + online theo QLCS</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Gói Camera cấu hình COD + online trên QLCS</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Phương thức thanh toán</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>Hiển thị COD "Thanh toán tại nhà" (kèm CTKM "Giảm trực tiếp 50% giá trị đơn hàng tối đa 200.000 VND") + các PTTT online theo QLCS; mỗi PTTT có badge ưu đãi (khác UltraFast: Camera CÓ COD). Cơ chế danh sách PTTT xem TC_CKCOMMON</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B19" s="22">
+        <f>IF(D19="","",$D$3&amp;"."&amp;COUNTA($D$10:D19)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Thông tin khách hàng auto-load + Thời gian lắp đặt</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>Đã nhập Thông tin cá nhân + Địa chỉ lắp đặt</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Thông tin khách hàng (cột phải)</t>
+        </is>
+      </c>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: "Thời gian lắp đặt" (vd Thứ 2, 02/01/2024 10:00-11:10) được set ở đâu/khi nào?]. Phần auto-load Họ tên/SĐT/Địa chỉ đúng theo dữ liệu đã nhập</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I19" s="25" t="n"/>
+      <c r="J19" s="25" t="n"/>
+      <c r="K19" s="25" t="n"/>
+      <c r="L19" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-CAMERA-001 (nguồn data Thời gian lắp đặt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 4: Button Thanh toán &amp; Luồng thanh toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B21" s="18">
+        <f>IF(D21="","",$D$3&amp;"."&amp;COUNTA($D$10:D21)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra Thanh toán khi chính sách không còn active trên QLCS</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>Gói/chính sách Camera không còn active trên QLCS</t>
+        </is>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>1. Click button "Thanh toán"</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>Báo lỗi chính sách không còn hiệu lực; KHÔNG thực hiện thanh toán</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B22" s="18">
+        <f>IF(D22="","",$D$3&amp;"."&amp;COUNTA($D$10:D22)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra Thanh toán khi data hợp lệ + chính sách active</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>Nhập đủ trường bắt buộc hợp lệ, chính sách active</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>1. Click button "Thanh toán"</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>Thực hiện luồng thanh toán theo PTTT đã chọn (COD → sang B3 luôn; Online → điều hướng cổng 3rd party)</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 5: Bước Hoàn tất đơn hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B24" s="18">
+        <f>IF(D24="","",$D$3&amp;"."&amp;COUNTA($D$10:D24)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hoàn tất đơn hàng với PTTT = COD</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>Chọn PTTT = COD, click Thanh toán</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>1. Hoàn tất đặt hàng với PTTT = COD
+2. Quan sát màn Hoàn tất</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>Màn Hoàn tất: trạng thái "Chưa thanh toán" + nội dung "Đơn hàng đã đăng ký thành công. Kỹ thuật viên FPT sẽ liên hệ triển khai dịch vụ trong 8h-12h. Mọi thắc mắc vui lòng liên hệ 1900 6600..."</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B25" s="18">
+        <f>IF(D25="","",$D$3&amp;"."&amp;COUNTA($D$10:D25)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hoàn tất đơn hàng với PTTT Online thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>Chọn PTTT Online, thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>1. Hoàn tất thanh toán Online thành công
+2. Quan sát màn Hoàn tất</t>
+        </is>
+      </c>
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>Bước "Hoàn tất đơn hàng" header màu xanh lá; trạng thái "Đã thanh toán" + nội dung thông báo thành công</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>IF(D26="","",$D$3&amp;"."&amp;COUNTA($D$10:D26)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra thanh toán Online thất bại quay về màn Thanh toán</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>Chọn PTTT Online, thanh toán thất bại</t>
+        </is>
+      </c>
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>1. Thực hiện thanh toán Online thất bại</t>
+        </is>
+      </c>
+      <c r="G26" s="20" t="inlineStr">
+        <is>
+          <t>Quay về màn Thanh toán giữ nguyên thông tin đã chọn; CHỈ cho thay đổi PTTT + nhập mã ưu đãi, các trường còn lại disable</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 6: Mã ưu đãi &amp; Hạng mục Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B28" s="22">
+        <f>IF(D28="","",$D$3&amp;"."&amp;COUNTA($D$10:D28)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra áp dụng mã ưu đãi / Chọn ưu đãi cho Camera</t>
+        </is>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán, có ô "Nhập mã khuyến mãi" + "Chọn ưu đãi"</t>
+        </is>
+      </c>
+      <c r="F28" s="24" t="inlineStr">
+        <is>
+          <t>1. Nhập mã ưu đãi / chọn ưu đãi
+2. Click "Áp dụng"</t>
+        </is>
+      </c>
+      <c r="G28" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: voucher/mã ưu đãi cho Camera chưa implement (như UltraFast SC-DANGKYUF-015)]. Kỳ vọng: trừ tiền vào "Cần thanh toán"</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I28" s="25" t="n"/>
+      <c r="J28" s="25" t="n"/>
+      <c r="K28" s="25" t="n"/>
+      <c r="L28" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-CAMAP-001 (voucher chưa implement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B29" s="22">
+        <f>IF(D29="","",$D$3&amp;"."&amp;COUNTA($D$10:D29)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra chọn loại địa chỉ Chung cư (radio Nhà riêng/Chung cư)</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Đang ở Block Địa chỉ lắp đặt</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>1. Chọn radio "Chung cư"</t>
+        </is>
+      </c>
+      <c r="G29" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – Deferred: Chung cư chưa phát triển ở version hiện tại (CLA-CKCOMMON-006), áp dụng chung mọi dịch vụ]</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I29" s="25" t="n"/>
+      <c r="J29" s="25" t="n"/>
+      <c r="K29" s="25" t="n"/>
+      <c r="L29" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED/Deferred – CLA-CKCOMMON-006 (Chung cư)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 7: Navigation &amp; Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B31" s="18">
+        <f>IF(D31="","",$D$3&amp;"."&amp;COUNTA($D$10:D31)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra button Quay lại điều hướng về màn Chi tiết gói</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Camera</t>
+        </is>
+      </c>
+      <c r="F31" s="20" t="inlineStr">
+        <is>
+          <t>1. Click button "Quay lại"</t>
+        </is>
+      </c>
+      <c r="G31" s="20" t="inlineStr">
+        <is>
+          <t>Điều hướng về màn Chi tiết gói Camera</t>
+        </is>
+      </c>
+      <c r="H31" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B32" s="18">
+        <f>IF(D32="","",$D$3&amp;"."&amp;COUNTA($D$10:D32)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị luồng Checkout Camera trên mobile (≤ 768px)</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>Mở checkout Camera trên viewport mobile</t>
+        </is>
+      </c>
+      <c r="F32" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát layout 2 bước + các block trên mobile</t>
+        </is>
+      </c>
+      <c r="G32" s="20" t="inlineStr">
+        <is>
+          <t>Các bước và block hiển thị đúng, không vỡ layout, thao tác được trên mobile</t>
+        </is>
+      </c>
+      <c r="H32" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B20:L20"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B9:L9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A3:L30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="3">
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Mã chức năng:</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>TC_AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Tên chức năng:</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Đăng ký dịch vụ Access Point (AP) — Checkout (số lượng + COD + địa chỉ lắp đặt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>QC/AI</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Testcase ID</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Mức Độ Ưu Tiên</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Nội Dung Test</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Điều Kiện / Dữ Liệu Test</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Các Bước Thực Hiện</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Kết Quả Mong Đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>Có thể
+Tự Động Hóa</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>Round 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>Kết Quả Thực Hiện</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>Người Thực Hiện</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>ID Bugs</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>Ghi Chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Lưu ý: Field validation (Họ tên, SĐT, Email, dropdown địa chỉ Tỉnh/Phường/Đường, popup Địa chỉ hành chính cũ, danh sách Phương thức thanh toán, luồng OTP) dùng chung — xem sheet Checkout_Common (TC_CKCOMMON). Sheet này chỉ kiểm tra phần ĐẶC THÙ dịch vụ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Lưu ý: AP giống Camera nhưng B1 CHỈ chọn số lượng (không có chu kỳ). Không có mockup riêng — tham chiếu layout mockup Camera (camera.png).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 1: Hiển thị &amp; Điều hướng vào Checkout (số lượng — không chu kỳ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <f>IF(D12="","",$D$3&amp;"."&amp;COUNTA($D$10:D12)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị tổng thể màn Checkout AP (2 bước)</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>Đã chọn gói AP ở màn Chi tiết</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát tiến trình và bố cục màn checkout AP</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Header 2 bước: "Thanh toán" → "Hoàn tất đơn hàng"; hiển thị đủ block: Sản phẩm dịch vụ đã chọn, Thông tin cá nhân, Địa chỉ lắp đặt, Phương thức thanh toán, Thông tin khách hàng, Thông tin thanh toán</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B13" s="22">
+        <f>IF(D13="","",$D$3&amp;"."&amp;COUNTA($D$10:D13)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra chọn số lượng (không chu kỳ) rồi Mua ngay sang Checkout</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>Ở màn Chi tiết gói AP</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>1. Chọn số lượng
+2. Click button "Mua ngay"</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: AP chỉ chọn số lượng, KHÔNG có chu kỳ?]. Kỳ vọng: điều hướng sang Thanh toán, load đúng tên gói + số lượng + số tiền</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I13" s="25" t="n"/>
+      <c r="J13" s="25" t="n"/>
+      <c r="K13" s="25" t="n"/>
+      <c r="L13" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-AP-001 (AP không chu kỳ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B14" s="22">
+        <f>IF(D14="","",$D$3&amp;"."&amp;COUNTA($D$10:D14)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Sản phẩm dịch vụ đã chọn (không hiển thị chu kỳ)</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán AP</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block "Sản phẩm dịch vụ đã chọn"</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: AP không có chu kỳ?]. Kỳ vọng: load đúng tên gói, số lượng, số tiền — KHÔNG hiển thị dòng chu kỳ</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I14" s="25" t="n"/>
+      <c r="J14" s="25" t="n"/>
+      <c r="K14" s="25" t="n"/>
+      <c r="L14" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-AP-001 (AP không chu kỳ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 2: Block Địa chỉ lắp đặt (đặc thù AP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B16" s="22">
+        <f>IF(D16="","",$D$3&amp;"."&amp;COUNTA($D$10:D16)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Địa chỉ lắp đặt + note giao hàng / Thời gian lắp đặt</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán AP</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Địa chỉ lắp đặt</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: AP có note giao hàng 3-7 ngày + Thời gian lắp đặt như Camera không?]. Phần fields địa chỉ (Tỉnh/Phường/Đường/Số nhà/Ghi chú + link địa chỉ cũ) xem TC_CKCOMMON</t>
+        </is>
+      </c>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I16" s="25" t="n"/>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="25" t="n"/>
+      <c r="L16" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-AP-002 (note giao hàng/Thời gian lắp đặt AP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 3: Phương thức thanh toán &amp; Thông tin khách hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B18" s="18">
+        <f>IF(D18="","",$D$3&amp;"."&amp;COUNTA($D$10:D18)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra AP CÓ phương thức COD + online theo QLCS</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Gói AP cấu hình COD + online trên QLCS</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Phương thức thanh toán</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>Hiển thị COD "Thanh toán tại nhà" + các PTTT online theo QLCS; chỉ chọn 1; "Xem thêm" nếu &gt;4. Cơ chế danh sách PTTT xem TC_CKCOMMON</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B19" s="22">
+        <f>IF(D19="","",$D$3&amp;"."&amp;COUNTA($D$10:D19)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Thông tin khách hàng auto-load</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>Đã nhập Thông tin cá nhân + Địa chỉ lắp đặt</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Thông tin khách hàng</t>
+        </is>
+      </c>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: AP có Thời gian lắp đặt không? (CLA-AP-002)]. Phần auto-load Họ tên/SĐT/Địa chỉ đúng theo dữ liệu đã nhập</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I19" s="25" t="n"/>
+      <c r="J19" s="25" t="n"/>
+      <c r="K19" s="25" t="n"/>
+      <c r="L19" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-AP-002 (Thời gian lắp đặt AP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 4: Button Thanh toán &amp; Luồng thanh toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B21" s="18">
+        <f>IF(D21="","",$D$3&amp;"."&amp;COUNTA($D$10:D21)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra Thanh toán khi chính sách không còn active trên QLCS</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>Gói/chính sách AP không còn active trên QLCS</t>
+        </is>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>1. Click button "Thanh toán"</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>Báo lỗi chính sách không còn hiệu lực; KHÔNG thực hiện thanh toán</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B22" s="18">
+        <f>IF(D22="","",$D$3&amp;"."&amp;COUNTA($D$10:D22)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra Thanh toán khi data hợp lệ + chính sách active</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>Nhập đủ trường bắt buộc hợp lệ, chính sách active</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>1. Click button "Thanh toán"</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>Thực hiện luồng thanh toán theo PTTT đã chọn (COD → sang B3 luôn; Online → cổng 3rd party)</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 5: Bước Hoàn tất đơn hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B24" s="18">
+        <f>IF(D24="","",$D$3&amp;"."&amp;COUNTA($D$10:D24)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hoàn tất đơn hàng với PTTT = COD</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>Chọn PTTT = COD, click Thanh toán</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>1. Hoàn tất đặt hàng với PTTT = COD
+2. Quan sát màn Hoàn tất</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>Màn Hoàn tất: trạng thái "Chưa thanh toán" + nội dung "Đơn hàng đã đăng ký thành công. Kỹ thuật viên FPT sẽ liên hệ triển khai dịch vụ trong 8h-12h..."</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B25" s="18">
+        <f>IF(D25="","",$D$3&amp;"."&amp;COUNTA($D$10:D25)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hoàn tất đơn hàng với PTTT Online thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>Chọn PTTT Online, thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>1. Hoàn tất thanh toán Online thành công
+2. Quan sát màn Hoàn tất</t>
+        </is>
+      </c>
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>Bước "Hoàn tất đơn hàng" header màu xanh lá; trạng thái "Đã thanh toán" + nội dung thông báo thành công</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>IF(D26="","",$D$3&amp;"."&amp;COUNTA($D$10:D26)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra thanh toán Online thất bại quay về màn Thanh toán</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>Chọn PTTT Online, thanh toán thất bại</t>
+        </is>
+      </c>
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>1. Thực hiện thanh toán Online thất bại</t>
+        </is>
+      </c>
+      <c r="G26" s="20" t="inlineStr">
+        <is>
+          <t>Quay về màn Thanh toán giữ nguyên thông tin đã chọn; CHỈ cho thay đổi PTTT + nhập mã ưu đãi, các trường còn lại disable</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Nhóm 6: Mã ưu đãi &amp; Navigation &amp; Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B28" s="22">
+        <f>IF(D28="","",$D$3&amp;"."&amp;COUNTA($D$10:D28)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr">
+        <is>
+          <t>Kiểm tra áp dụng mã ưu đãi cho AP</t>
+        </is>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán AP</t>
+        </is>
+      </c>
+      <c r="F28" s="24" t="inlineStr">
+        <is>
+          <t>1. Nhập/áp dụng mã ưu đãi</t>
+        </is>
+      </c>
+      <c r="G28" s="24" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: voucher/mã ưu đãi chưa implement (như UltraFast)]. Kỳ vọng: trừ tiền</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I28" s="25" t="n"/>
+      <c r="J28" s="25" t="n"/>
+      <c r="K28" s="25" t="n"/>
+      <c r="L28" s="24" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-CAMAP-001 (voucher chưa implement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B29" s="18">
+        <f>IF(D29="","",$D$3&amp;"."&amp;COUNTA($D$10:D29)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra button Quay lại điều hướng về màn Chi tiết gói</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán AP</t>
+        </is>
+      </c>
+      <c r="F29" s="20" t="inlineStr">
+        <is>
+          <t>1. Click button "Quay lại"</t>
+        </is>
+      </c>
+      <c r="G29" s="20" t="inlineStr">
+        <is>
+          <t>Điều hướng về màn Chi tiết gói AP</t>
+        </is>
+      </c>
+      <c r="H29" s="18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B30" s="18">
+        <f>IF(D30="","",$D$3&amp;"."&amp;COUNTA($D$10:D30)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị luồng Checkout AP trên mobile (≤ 768px)</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>Mở checkout AP trên viewport mobile</t>
+        </is>
+      </c>
+      <c r="F30" s="20" t="inlineStr">
+        <is>
+          <t>1. Quan sát layout 2 bước + các block trên mobile</t>
+        </is>
+      </c>
+      <c r="G30" s="20" t="inlineStr">
+        <is>
+          <t>Các bước và block hiển thị đúng, không vỡ layout, thao tác được trên mobile</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B15:L15"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B20:L20"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B9:L9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>